<commit_message>
Add Min N and No3 analyses
</commit_message>
<xml_diff>
--- a/Tables/aicc_tables.xlsx
+++ b/Tables/aicc_tables.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Analysis_2_POM_C_N" sheetId="2" r:id="rId2"/>
     <sheet name="Analysis_3_Microbial_biomass" sheetId="3" r:id="rId3"/>
     <sheet name="Analysis_4_pH_cations" sheetId="4" r:id="rId4"/>
+    <sheet name="Analysis_6_Mineral_N" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2574,4 +2575,170 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Response/Hypothesis</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>AICc</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Δi</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ωi</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Evid. ratio</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Model Formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>tot_min_n_ha</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quadratic</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>78</v>
+      </c>
+      <c r="E2">
+        <v>0.65</v>
+      </c>
+      <c r="F2">
+        <v>832.1</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>months² × treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Square Root</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>78</v>
+      </c>
+      <c r="E3">
+        <v>0.57</v>
+      </c>
+      <c r="F3">
+        <v>843.3</v>
+      </c>
+      <c r="G3">
+        <v>11.2</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>276.92</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>sqrt(months) × treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Linear</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>78</v>
+      </c>
+      <c r="E4">
+        <v>0.55</v>
+      </c>
+      <c r="F4">
+        <v>847.2</v>
+      </c>
+      <c r="G4">
+        <v>15.1</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>1902.91</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>months × treatment</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>